<commit_message>
Leads: 2026-09-13 04:17 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://northcreekroofing.com/areas-served/olympia/</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>info@northcreekroofing.com</t>
@@ -614,6 +613,186 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hail Belt Roofing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>hailbeltroofing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.hailbeltroofing.com/abilene-tx/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Hail Belt</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>leads@hailbeltroofing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(888) 814-2837</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>roof replacement Abilene TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Roof Replacement Abilene</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>roofreplacementabilene.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://roofreplacementabilene.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Roof Replacement</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@roofreplacementabilene.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>325-268-5560</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roof replacement Abilene TX</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Top Roofing Company in Abilene, TX | Roof Repair</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>satisfactionsolutions.net</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://satisfactionsolutions.net/roofing/abilene-tx</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Roof Repair</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>hi@satisfactionsolutions.net</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>682-332-9709</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roof replacement Abilene TX</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:21 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,126 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>My Happy Home</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>myhappyhome.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://myhappyhome.com/hvac/heat-pump-installation-replacement-nashville-tn</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Happiness We</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>support@myhappyhome.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(855) 797-6944</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>heat pump installation Nashville TN</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Webster Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>websterac.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://websterac.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Air Filters</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info@websterac.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(407) 295-0598</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>96</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HVAC contractor Orlando FL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:22 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,122 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Harris Roofing - Expert Roofing Services in Anchorage, AK</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>harrisroofingalaska.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://harrisroofingalaska.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>scheduling@harrisroofingalaska.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1206401760</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof replacement Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Black Spruce Roofing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>blackspruceroofing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://blackspruceroofing.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Checked Crew</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>blackspruceroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(907) 416-5802</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roof replacement Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:27 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -939,7 +939,6 @@
           <t>https://harrisroofingalaska.com/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>scheduling@harrisroofingalaska.com</t>
@@ -1029,6 +1028,474 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Big Red Contracting</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>bigredcontractingky.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://bigredcontractingky.com/roof-replacement-lexington-ky/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Owner Claim</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@bigredcontractingky.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(502) 395-8804</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roof replacement Lexington KY</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Roof Replacement | Lexington, KY</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>kentuckyhomeservicesky.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.kentuckyhomeservicesky.com/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>kentuckyhomeservices@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(859) 621-3257</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roof replacement Lexington KY</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Plumber In Surprise AZ | The Family Plumber | Arizona Plumbing Company</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>callthefamilyplumber.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.callthefamilyplumber.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@callthefamilyplumber.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(623) 738-6171</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Surprise AZ</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>water heater repair Surprise AZ</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ray Gidich Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>raygidich.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.raygidich.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>contact@raygidich.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(440) 245-1772</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Lorain OH</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>air conditioning repair Lorain OH</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Reliable Water Heater Repair in Surprise, AZ</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>highspeedplumbingaz.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.highspeedplumbingaz.com/water-heater-repair-replacement-surprise-az</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Shower Repair</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>highspeedplumbingaz@gmail.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>480-572-4290</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Surprise AZ</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>water heater repair Surprise AZ</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair in Lorain, OH | AC Repair | Stack</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>stackheating.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://stackheating.com/air-conditioning-repair/lorain-oh/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>History Request</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@stackheating.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(440) 937-9134</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Lorain OH</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>air conditioning repair Lorain OH</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Truetemp HVAC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>truetemphvac.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://truetemphvac.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>truetemp@truetemphvac.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>409-571-3333</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Beaumont TX</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>heating and cooling company Beaumont TX</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Reed Service Company</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>reedservice.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>http://reedservice.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Protect My</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>reedservice@reedservice.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(409) 842-0336</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Beaumont TX</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>88</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>heating and cooling company Beaumont TX</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:28 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1114,7 +1114,6 @@
           <t>https://www.kentuckyhomeservicesky.com/roof-replacement</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>kentuckyhomeservices@gmail.com</t>
@@ -1170,7 +1169,6 @@
           <t>https://www.callthefamilyplumber.com/water-heater-repair/</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>info@callthefamilyplumber.com</t>
@@ -1226,7 +1224,6 @@
           <t>https://www.raygidich.com/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>contact@raygidich.com</t>
@@ -1496,6 +1493,126 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hellenic Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>hellenicroofing.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://hellenicroofing.com/pasadena-tx/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Comprehensive Commercial</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>hellenicroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(832) 704-2817</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>residential roofing company Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Upstanding Roofing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>upstandingroofing.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.upstandingroofing.com/service-areas/pasadena-tx/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Ben Pacheco</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>sales@upstandingroofing.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(833) 390-3730</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>86</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>residential roofing company Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:30 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1618,6 +1618,182 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Milwaukee Roof Repair Pros</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>milwaukeeroofrepairpros.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://milwaukeeroofrepairpros.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>All Rights</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>hi@milwaukeeroofrepairpros.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>877 499 2535</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Milwaukee WI</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roof repair company Milwaukee WI</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Schwantes Heating and Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>schwantesheating.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://schwantesheating.com/ac-installation-bloomington-mn-39764/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>info@schwantesheating.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>651-439-3331</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Bloomington MN</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>AC installation Bloomington MN</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pioneershvacsc.com</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>pioneershvacsc.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://pioneershvacsc.com/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Santa Clarita</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>info@pioneershvacsc.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(661) 238-4148</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>heating and cooling company Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:31 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1699,7 +1699,6 @@
           <t>https://schwantesheating.com/ac-installation-bloomington-mn-39764/</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>info@schwantesheating.com</t>
@@ -1789,6 +1788,238 @@
         </is>
       </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Strategic Roofing</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>strategic-roofers.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://strategic-roofers.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Pinellas Park</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>office@strategic-roofers.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>727-442-7663</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>roofer Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Roofer Clearwater</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>drrooferclearwater.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://drrooferclearwater.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>cs@drrooferflorida.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(727) 233-5289</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>roofer Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>A1 Air Conditioning &amp; Heating LLC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>a1airconditioningtucson.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://a1airconditioningtucson.com/tucson-az-hvac-contractor/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Air Conditioning</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>web@lmh.agency</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(520) 704-7208</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>90</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Arizona Daily Star</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>tucson.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://tucson.com/exclusive/article_52429529-0b1c-54da-9aba-31959ab88ba9.html</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>mobile@tucson.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(800)695-4492</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>84</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:33 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1874,7 +1874,6 @@
           <t>https://drrooferclearwater.com/</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>cs@drrooferflorida.com</t>
@@ -1990,7 +1989,6 @@
           <t>https://tucson.com/exclusive/article_52429529-0b1c-54da-9aba-31959ab88ba9.html</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>mobile@tucson.com</t>
@@ -2020,6 +2018,66 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Proactive Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>proactiveairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://proactiveairconditioning.com/air-conditioner-installation-replacement-dallas-tx/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Prioritize Customers</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>info@proactiveairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(469) 921-1136</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>AC installation Dallas TX</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:34 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2083,6 +2083,62 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Premier Cooling LLC</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>premiercoolingllc.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://premiercoolingllc.com/location/miramar/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>premiercoolingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>954-257-9998</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>heating and cooling company Miramar FL</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:37 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2104,7 +2104,6 @@
           <t>https://premiercoolingllc.com/location/miramar/</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>premiercoolingllc@gmail.com</t>
@@ -2134,6 +2133,66 @@
         </is>
       </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HVAC Company New Jersey</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>heat-pump-installation-woodbridge.aeshvacnj.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://heat-pump-installation-woodbridge.aeshvacnj.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>example@mail.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(888) 978-1291</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>100</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>heat pump installation Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:42 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2198,6 +2198,122 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Athens &amp; Augusta GA | Georgia Best Roofing</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>georgiabestroofing.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://georgiabestroofing.com/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>georgiabestroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(706)-975-6103</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Athens GA</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Athens GA</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Boise, Idaho HVAC Company - Snowflake Air | We’re Not Comfortable Until You Are</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>snowflakeair.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://snowflakeair.com/meridian-id-heat-pump/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Cleaning Worry</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>info@snowflakeair.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(208) 205-9078</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Meridian ID</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>heat pump installation Meridian ID</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:43 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2219,7 +2219,6 @@
           <t>https://georgiabestroofing.com/services/metal-roofing</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>georgiabestroofing@gmail.com</t>
@@ -2309,6 +2308,66 @@
         </is>
       </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Plumber Waco Texas</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>plumberwacotx.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://plumberwacotx.com/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Fixture Installation</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>mubeenshahjahan0@gmail.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(254) 489-8427</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Waco TX</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>plumber Waco TX</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:45 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2373,6 +2373,122 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Birdwell AC &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>birdwellacandheating.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://birdwellacandheating.com/furnace-repair-corpus-christi-tx/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>birdwellair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(361) 452-2018</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>100</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>furnace repair Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Swift Air</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>swiftaircc.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.swiftaircc.com/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Team May</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>service@swiftaircc.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>361-882-2111</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>furnace repair Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:46 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2394,7 +2394,6 @@
           <t>https://birdwellacandheating.com/furnace-repair-corpus-christi-tx/</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>birdwellair@gmail.com</t>
@@ -2484,6 +2483,66 @@
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Thermal-Tech Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>thermal-techohio.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.thermal-techohio.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Everyone Like</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(330) 484-6579</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Canton OH</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>HVAC contractor Canton OH</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:55 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2548,6 +2548,62 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Eades Heating &amp; Cooling – Springfield, Illinois</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>eadesheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://eadesheatingandair.com/heating/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>eadesemail@gmail.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>217-529-5767</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Springfield IL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>98</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>furnace repair Springfield IL</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:57 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2569,7 +2569,6 @@
           <t>https://eadesheatingandair.com/heating/</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>eadesemail@gmail.com</t>
@@ -2599,6 +2598,302 @@
         </is>
       </c>
       <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AAP Air Conditioning and Heating Repair</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>aapair.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.aapair.com/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>contact@aapair.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>941-312-6253</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>100</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>air conditioning repair Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>The Hennessy Group</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>thehennessygrp.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.thehennessygrp.com/warwick-ri-plumbers</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Plumbing Services</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@thehennessygrp.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>401.736.8300</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Warwick RI</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>plumber Warwick RI</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Streamline Heating and Air - Streamline Air A/C</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>streamlineairfl.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://streamlineairfl.com/air-conditioner-repair-sarasota/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Air Conditione</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>office.streamlineac@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>941-356-6872</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>100</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>air conditioning repair Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>My Blog</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>roundrockdraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://roundrockdraincleaning.com/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>info@roundrockdraincleaning.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(737) 775-7412</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>94</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>drain cleaning service Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Infinity Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>infinityairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.infinityairconditioning.com/locations/sarasota</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Why North</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>office@infinityairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>941-876-3788</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>air conditioning repair Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 04:58 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2624,7 +2624,6 @@
           <t>https://www.aapair.com/</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>contact@aapair.com</t>
@@ -2894,6 +2893,66 @@
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Farwest</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>farwestclimatecontrol.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.farwestclimatecontrol.com/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Burt Ross</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>office@farwestclimatecontrol.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(509) 457-5346</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Yakima WA</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>88</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>heating and cooling company Yakima WA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:00 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2958,6 +2958,66 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Roof Repair &amp; Replacement Services in Savannah, GA</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>savannah-ga.guyroofingcoinc.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://savannah-ga.guyroofingcoinc.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Guy Roofing</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>info@guyroofingcoinc.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(770) 727-3408</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Savannah GA</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>90</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>roof repair company Savannah GA</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:01 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3018,6 +3018,66 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>The Local Guys</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>localguysplumbing.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://localguysplumbing.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Why Spokane</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>localguysplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>509-808-0713</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>100</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>drain cleaning service Spokane WA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:04 UTC (cycle 34)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3078,6 +3078,66 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Axis Remodeling</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>axisremodeling.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://axisremodeling.com/roofing/wi/winnebago-county/oshkosh/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Oshkosh Homeowners</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>contact@axisremodeling.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(920) 278-3123</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Oshkosh WI</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>90</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>roof replacement Oshkosh WI</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:05 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3138,6 +3138,66 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Residential Roofing Services Syracuse NY</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>syracuseexteriors.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.syracuseexteriors.com/residential-roofing.html</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Communities Based</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@syracuseexteriors.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>315-273-2973</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Syracuse NY</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>residential roofing company Syracuse NY</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:11 UTC (cycle 39)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3198,6 +3198,66 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SoCal Emergency Plumbing Los Angeles</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>socalemergencyplumbinglosangeles.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://socalemergencyplumbinglosangeles.com/service-areas/irvine</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Southern California</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>info@socalemergencyplumbinglosangeles.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(213) 660-7353</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>90</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>emergency plumber Irvine CA</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:14 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3258,6 +3258,298 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>THE PLUMBING POLICE MIAMI</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>plumbingpolicemiami.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://plumbingpolicemiami.com/24-hour-emergency</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>info@indiantypefoundry.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(305) 834-0511</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>emergency plumber Miami FL</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Miami Plumbers 24-hr Emergency Services | High End Plumbing</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>miamiemergencyplumbing.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.miamiemergencyplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Miami Homeowners</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>mep@miamiemergencyplumbing.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(305) 501-2093</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>100</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>emergency plumber Miami FL</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>localhomeplumbers.com</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>localhomeplumbers.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://localhomeplumbers.com/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>wasiimlatiif142@gmail.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(305) 786-4811</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>emergency plumber Miami FL</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Plumbers Miami Florida</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>plumberinmiamiflorida.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://plumberinmiamiflorida.com/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Emergency Ready</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>plumberinmiamiflorida@gmail.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(305) 404-5531</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>90</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>emergency plumber Miami FL</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Wyn Miami Plumbing</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>emergencyplumbermiamifl.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://emergencyplumbermiamifl.com/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Little Havana</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>wynmiamiplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(305) 630-8680</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>emergency plumber Miami FL</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:17 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3279,7 +3279,6 @@
           <t>https://plumbingpolicemiami.com/24-hour-emergency</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>info@indiantypefoundry.com</t>
@@ -3395,7 +3394,6 @@
           <t>https://localhomeplumbers.com/</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>wasiimlatiif142@gmail.com</t>
@@ -3545,6 +3543,62 @@
         </is>
       </c>
       <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Metal Roofing Services in Gresham, OR | Columbia Gorge Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>columbiagorgesheetmetal.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://columbiagorgesheetmetal.com/service-areas/gresham-or</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>etal@gmail.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>5416454845</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Gresham OR</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>82</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Gresham OR</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:25 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3569,7 +3569,6 @@
           <t>https://columbiagorgesheetmetal.com/service-areas/gresham-or</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>etal@gmail.com</t>
@@ -3599,6 +3598,66 @@
         </is>
       </c>
       <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Roofing Company in Hialeah, FL | Roof Repair &amp; Replacement</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>orianroofingmia.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://orianroofingmia.com/service-areas/hialeah/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Orian Roofing</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>orianroofingmia@gmail.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(305) 707-4457</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>100</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>roof replacement Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:29 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3663,6 +3663,66 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Grand Rapids Residential &amp; Commercial Plumber | NSP Plumbing</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>needsomeplumbing.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.needsomeplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>West Michigan</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>info@needsomeplumbing.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(616) 207-9960</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>100</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>plumbing company Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:33 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3723,6 +3723,62 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Hot and Flow Services</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>hotandflow.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://hotandflow.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>anthony@hotandflow.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>272-207-8047</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Scranton PA</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>74</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>drain cleaning service Scranton PA</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:46 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3744,7 +3744,6 @@
           <t>https://hotandflow.com/services/drain-cleaning/</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>anthony@hotandflow.com</t>
@@ -3774,6 +3773,66 @@
         </is>
       </c>
       <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Perfect Home Services -</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>perfecthomeservices.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://www.perfecthomeservices.com/plumbing/water-heater/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Addison Bensenville</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>clientcare@www.perfecthomeservices.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>630-216-4926</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Aurora IL</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>90</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>water heater repair Aurora IL</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:48 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3838,6 +3838,66 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>infinityservicesar.com</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>infinityservicesar.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://infinityservicesar.com/ac-repair-little-rock-ar/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>North Little</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>info@infinityservicesar.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(501) 299-3167</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>90</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>air conditioning repair Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:52 UTC (cycle 67)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3898,6 +3898,62 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Roof Replacement | Bethlehem, PA | Roofing By Bruce</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>roofingbybruce.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.roofingbybruce.com/sap/roof-replacement/bethlehem-pa</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>info@roofingbybruce.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(570) 203-2142</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>roof replacement Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 05:54 UTC (cycle 68)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3919,7 +3919,6 @@
           <t>https://www.roofingbybruce.com/sap/roof-replacement/bethlehem-pa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>info@roofingbybruce.com</t>
@@ -3949,6 +3948,62 @@
         </is>
       </c>
       <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Lunas Roofing</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>lunas-roofing.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://lunas-roofing.com/fresno-ca/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>lunasroofing1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(209) 720-9974</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>90</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>residential roofing company Fresno CA</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:01 UTC (cycle 73)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3974,7 +3974,6 @@
           <t>https://lunas-roofing.com/fresno-ca/</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>lunasroofing1@gmail.com</t>
@@ -4004,6 +4003,62 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Syracuse, NY Roofing Services | TopTier Roofing</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>toptierroofingcny.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.toptierroofingcny.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>info@toptierroofingcny.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(315) 877-3760</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Syracuse NY</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>86</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>roofer Syracuse NY</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:03 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4029,7 +4029,6 @@
           <t>https://www.toptierroofingcny.com/</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>info@toptierroofingcny.com</t>
@@ -4059,6 +4058,62 @@
         </is>
       </c>
       <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>A-C Air Care</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>acaircare.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.acaircare.com/service-areas/columbia-md/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>jaime@acaircare.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>410-220-0503</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Columbia MD</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>100</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>air conditioning repair Columbia MD</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:04 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4084,7 +4084,6 @@
           <t>https://www.acaircare.com/service-areas/columbia-md/ac-repair/</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>jaime@acaircare.com</t>
@@ -4114,6 +4113,62 @@
         </is>
       </c>
       <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Plumbers Toledo, OH | Drain Doctor</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>toledoplumbingcompany.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.toledoplumbingcompany.com/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>draindoctoroffice@bex.net</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(419) 314-3820</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>100</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>plumbing company Toledo OH</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:06 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4139,7 +4139,6 @@
           <t>https://www.toledoplumbingcompany.com/</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>draindoctoroffice@bex.net</t>
@@ -4169,6 +4168,66 @@
         </is>
       </c>
       <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Sewer Studs</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>sewerstuds.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://www.sewerstuds.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Tampa Bay</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>info@sewerstuds.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>813-680-2284</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>90</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>drain cleaning service Tampa FL</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:07 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4233,6 +4233,126 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Omaha, NE</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>omahafreshair.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://omahafreshair.com/services/heat-pumps</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Ryan Cartwright</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>omahafreshair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>402-515-9164</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>90</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>heat pump installation Omaha NE</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>sunsetair</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>sunsetcooling.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.sunsetcooling.com/irvine</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Abe Fierro</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>sunset-air@outlook.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(949) 302-3473</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>90</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>heating and cooling company Irvine CA</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:21 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4353,6 +4353,66 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>75 Degree AC</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>75degreeac.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://75degreeac.com/services/furnace-repair-houston/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Easy Scheduling</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>info@75degreeac.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(713) 598-2737</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>90</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>furnace repair Houston TX</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:22 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4413,6 +4413,62 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Pueblo</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>draperheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://draperheatingandairconditioning.com/locations/pueblo-co/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>info@draperheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(888) 919-5064</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Pueblo CO</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>90</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>heat pump installation Pueblo CO</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:27 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4434,7 +4434,6 @@
           <t>https://draperheatingandairconditioning.com/locations/pueblo-co/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>info@draperheatingandairconditioning.com</t>
@@ -4464,6 +4463,126 @@
         </is>
       </c>
       <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Roof Repair in Waldorf, MD | All Purpose Anytime Services</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>allpurposeanytimeservices.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.allpurposeanytimeservices.com/services/roof-repair-waldorf-md</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Area Drywall</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>hello@allpurposeanytimeservices.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(240) 695-4415</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Waldorf MD</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>100</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>roof repair company Waldorf MD</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Cook's Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>cookshc.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://cookshc.com/heating-cooling-winston-salem-nc/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Know Facts</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>info@cookshc.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(336) 969-6576</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>100</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>heating and cooling company Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:30 UTC (cycle 92)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4588,6 +4588,122 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Anytime Drain Cleaning Sewer Repair and Pipelining</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>albuquerquedrainsewerpipeline.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://albuquerquedrainsewerpipeline.com/services/albuquerque-drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>info@albuquerquedrainsewerpipeline.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>(505) 474-4441</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>drain cleaning service Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Best Roofers Acworth Ga | Bravo Company Roofing - Roofing Services in Atlanta an</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>bravoroof.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://bravoroof.com/marietta-ga-roofing/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Shane Ferraro</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>info@bravoroof.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>404.783.5785</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>roof replacement Marietta GA</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:32 UTC (cycle 94)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4609,7 +4609,6 @@
           <t>https://albuquerquedrainsewerpipeline.com/services/albuquerque-drain-cleaning/</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>info@albuquerquedrainsewerpipeline.com</t>
@@ -4699,6 +4698,66 @@
         </is>
       </c>
       <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Beaverton Roofing Company | Repairs, Reroofs, &amp; Installs</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>redbirdroofs.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.redbirdroofs.com/service-areas/beaverton-or</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Book Now</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>joe@redbirdroofs.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(360) 605-3127</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Beaverton OR</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>90</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>roof repair company Beaverton OR</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:41 UTC (cycle 100)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4763,6 +4763,238 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Metal Roofing Contractor | Winston-Salem, NC | B&amp;M Roofing Contractors</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>bmroofingcontractors.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.bmroofingcontractors.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>sgreer@bmroofingcontractors.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>252-442-5300</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>100</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Metal Roofing | Best Roofing of Winston Salem</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>bestroofingofws.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.bestroofingofws.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>What We</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>sales@bestroofingofws.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(336) 407-6155</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Roofing Brothers</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>roofingbrothersinc.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.roofingbrothersinc.com/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Sherwood Forest</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>info@roofingbrothersinc.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(336) 701-0075</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>90</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Metal Roof Winston Salem</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>metalroofwinstonsalem.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>http://www.metalroofwinstonsalem.com/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofwinstonsalem.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>866-868-1006</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>84</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:44 UTC (cycle 102)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4784,7 +4784,6 @@
           <t>https://www.bmroofingcontractors.com/metal-roofing</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>sgreer@bmroofingcontractors.com</t>
@@ -4960,7 +4959,6 @@
           <t>http://www.metalroofwinstonsalem.com/</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>moreinfo@metalroofwinstonsalem.com</t>
@@ -4990,6 +4988,66 @@
         </is>
       </c>
       <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Ellis Air Systems | HVAC repairs and installs | Killeen and Temple TX</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ellisairsystems.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.ellisairsystems.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Cooling Our</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>info@ellisairsystems.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(254) 526-5410</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Killeen TX</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>98</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>air conditioning repair Killeen TX</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:55 UTC (cycle 109)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5053,6 +5053,66 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Lancaster, PA - George J. Grove &amp; Son</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>georgejgrove.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.georgejgrove.com/roofing/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Manheim Pike</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>info@georgejgrove.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>717.393.0859</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>100</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>roofing contractor Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:56 UTC (cycle 110)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5113,6 +5113,178 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>BIG RED ROOFING &amp; Home Exteriors</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>bigred-roofing.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://bigred-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>info@bigred-roofing.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>(919) 441-2735</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Cary NC</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>100</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>residential roofing company Cary NC</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>My Blog</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>waterheaterlco.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://waterheaterlco.com/areas-we-serve/arvada/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>support@waterheaterlco.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(201) 277-9344</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>92</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>water heater repair Arvada CO</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Mile High Plumbing, Electric &amp; Air</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>milehighmep.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://www.milehighmep.com/water-heater-repair-arvada-co</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Career Services</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>service@milehighmep.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>303) 859-0100</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>90</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>water heater repair Arvada CO</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:58 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5134,7 +5134,6 @@
           <t>https://bigred-roofing.com/</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>info@bigred-roofing.com</t>
@@ -5190,7 +5189,6 @@
           <t>https://waterheaterlco.com/areas-we-serve/arvada/</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>support@waterheaterlco.com</t>
@@ -5280,6 +5278,126 @@
         </is>
       </c>
       <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Roof Replacement | Las Vegas, NV</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>discountroofingnv.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.discountroofingnv.com/roof-replacement-las-vegas-nv</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Southern Nevada</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>discountroofingnv@gmail.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>702-355-8287</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>90</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>roof replacement Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>YMC Inc. Mechanical Contractor</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>ymcinc.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://ymcinc.com/air-conditioning-repair-boise-id-601871/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Comprehensive Residential</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>information@ymcinc.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(208) 634-2859</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>90</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>air conditioning repair Boise ID</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 06:59 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5403,6 +5403,62 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Done Right Plumbing</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>drplv.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.drplv.com/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>service@drplv.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>702-940-5352</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Henderson NV</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>94</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>sewer repair Henderson NV</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:07 UTC (cycle 117)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5424,7 +5424,6 @@
           <t>https://www.drplv.com/</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>service@drplv.com</t>
@@ -5454,6 +5453,178 @@
         </is>
       </c>
       <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>AC Installation | Whole-House Cooling | Honolulu, HI</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>airsourceac.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.airsourceac.com/ac-installation</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>airsourceac@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(808) 300-4651</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>100</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>AC installation Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Air Conditioning Installation Honolulu HI | American AC</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>americanachawaii.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.americanachawaii.com/ac-installation-honolulu-hi</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Why Honolulu</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>americanairconditioninghawaii@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(808)-847-0851</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>94</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>AC installation Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>A/C Installation | Honolulu, HI | Advanced A/C Contracting</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>advancedachawaii.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.advancedachawaii.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>info@advancedachawaii.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>808-847-4814</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>84</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>AC installation Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:08 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5479,7 +5479,6 @@
           <t>https://www.airsourceac.com/ac-installation</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>airsourceac@yahoo.com</t>
@@ -5595,7 +5594,6 @@
           <t>https://www.advancedachawaii.com/</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>info@advancedachawaii.com</t>
@@ -5625,6 +5623,182 @@
         </is>
       </c>
       <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Fort Collins Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>severeweatherroofing.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://severeweatherroofing.com/fort-collins-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>John Anderson</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>home@severeweatherroofing.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>970-223-2455</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>90</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Metal Roofing - HD Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>hdroofingcolorado.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://hdroofingcolorado.com/metal-roofing-fort-collins-co</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Fort Collins</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>info@hdroofingcolorado.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(970) 823-8103</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>88</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Fort Collins, CO</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>peterichcustomconstruction.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://peterichcustomconstruction.com/metal</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Dan Peterich</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>team@latofonts.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>76</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:14 UTC (cycle 122)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5779,7 +5779,6 @@
           <t>team@latofonts.com</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>Fort Collins CO</t>
@@ -5799,6 +5798,62 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Best Roofing Contractor in Bellingham, WA | Esary Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>esary.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.esary.com/bellingham--wa-residential-roofing-contractor</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>info@esary.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(360) 757-0933</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>90</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>roof replacement Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:17 UTC (cycle 124)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5824,7 +5824,6 @@
           <t>https://www.esary.com/bellingham--wa-residential-roofing-contractor</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>info@esary.com</t>
@@ -5854,6 +5853,66 @@
         </is>
       </c>
       <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>East NYC Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>eastnycroofing.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://eastnycroofing.com/</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>What We</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>nick@eastnycroofing.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>917-900-0555</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>100</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>roofing contractor Queens NY</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:26 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5918,6 +5918,66 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Marietta Plumbing Experts</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>plumbingcompanymarietta.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://plumbingcompanymarietta.com/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Cobb County</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>service@plumbingcompanymarietta.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(770) 588-0267</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>90</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>plumbing company Marietta GA</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:29 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5978,6 +5978,126 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Roof Replacement Austin TX | Residential Roofing | Austin Roofers</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>austinroofer.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://austinroofer.com/residential-roofing/replacement</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Why Austin</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>info@austinroofer.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(512) 764-3547</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>100</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>roof replacement Austin TX</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Marietta Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>mariettametalroofing.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://mariettametalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Message From</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>go@ccteam.org</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(864) 259-1707</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>100</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Marietta GA</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:30 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6098,6 +6098,122 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Charlotte NC | Open Water Plumbing</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>openwaterplumbing.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.openwaterplumbing.com/water-heater-repair-charlotte-nc</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>info@openwaterplumbing.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>980-613-1572</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Charlotte NC</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>100</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>water heater repair Charlotte NC</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Evergreen Providence — Comfortable today. Sustainable tomorrow.</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>evergreenprovidence.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://evergreenprovidence.com/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>hello@evergreenprovidence.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(971) 449-1058</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Providence RI</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>100</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>heat pump installation Providence RI</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:32 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6119,7 +6119,6 @@
           <t>https://www.openwaterplumbing.com/water-heater-repair-charlotte-nc</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>info@openwaterplumbing.com</t>
@@ -6209,6 +6208,66 @@
         </is>
       </c>
       <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Will's Plumbing &amp; Testing Service</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>willsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://willsplumbing.com/new-braunfels-tx/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Office Will</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>info@willsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(210) 494-0991</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>90</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>plumber New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:36 UTC (cycle 137)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6273,6 +6273,62 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Precision Roofing Services Co</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>precisionroofingservicesco.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://precisionroofingservicesco.com/metal-roofing-services</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>services@precisionroofingservicesco.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(785) 377-6233</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Lawrence KS</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>90</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lawrence KS</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:38 UTC (cycle 138)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6294,7 +6294,6 @@
           <t>https://precisionroofingservicesco.com/metal-roofing-services</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>services@precisionroofingservicesco.com</t>
@@ -6324,6 +6323,62 @@
         </is>
       </c>
       <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair | Toledo, OH | Air-Stream Plumbing Heating Cooling</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>airstreamplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.airstreamplumbingheating.com/air-conditioning-repair/toledo-oh</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>airstreamplumbingheating@gmail.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(419) 825-2364</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>90</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>air conditioning repair Toledo OH</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:42 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6349,7 +6349,6 @@
           <t>https://www.airstreamplumbingheating.com/air-conditioning-repair/toledo-oh</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>airstreamplumbingheating@gmail.com</t>
@@ -6379,6 +6378,66 @@
         </is>
       </c>
       <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Drain Pros</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>drainprosventura.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://drainprosventura.com/santa-clarita-ca/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Plumber Drain</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>jesse@drainprosventura.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>805-791-3954</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>100</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>drain cleaning service Santa Clarita CA</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:45 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6443,6 +6443,62 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Sugar Land TX Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>sugarlanddraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://sugarlanddraincleaning.com/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>service@sugarlanddraincleaning.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>281-940-4091</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>100</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>drain cleaning service Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:48 UTC (cycle 145)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6464,7 +6464,6 @@
           <t>https://sugarlanddraincleaning.com/</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>service@sugarlanddraincleaning.com</t>
@@ -6494,6 +6493,66 @@
         </is>
       </c>
       <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Residential &amp; Commercial HVAC — Kent, WA | Coast Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>coastheatandair.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://www.coastheatandair.com/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>South King</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>office@coastheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(206) 920-5547</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Kent WA</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>90</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>heating and cooling company Kent WA</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:55 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6558,6 +6558,66 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>HVAC Contractor | Greenville, South Carolina | Grace Services of the Upstate LLC</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>graceheatingandairservices.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.graceheatingandairservices.com/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Customer Service</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>cliff@graceheatingandairservices.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>864-775-6209</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>90</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>HVAC contractor Greenville SC</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 07:58 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6618,6 +6618,62 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Metal Roof Hollywood</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>metalroofhollywood.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>http://metalroofhollywood.com/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofhollywood.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>866-868-1006</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>84</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:04 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6639,7 +6639,6 @@
           <t>http://metalroofhollywood.com/</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>moreinfo@metalroofhollywood.com</t>
@@ -6669,6 +6668,66 @@
         </is>
       </c>
       <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair Mount Pleasant &amp; Charleston, SC | Water Heater Doctors</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>waterheaterdocs.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://waterheaterdocs.com/sewer-line-services</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Mount Pleasant</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>info@waterheaterdocs.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(843) 990-6524</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Mount Pleasant SC</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>90</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>sewer repair Mount Pleasant SC</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:06 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6733,6 +6733,66 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Local Roofing Contractor Germantown, MD</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>kcconstructionroofing.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://kcconstructionroofing.com/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Siding Services</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@kcconstructionroofing.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(240) 358-0873</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Germantown MD</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>90</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>roofing contractor Germantown MD</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:10 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6793,6 +6793,62 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CandelTech Services</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>candeltechservices.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://candeltechservices.com/hvac-contractor-carrollton-tx/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>services@candeltechservices.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>817-616-3405</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>90</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>HVAC contractor Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:12 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6814,7 +6814,6 @@
           <t>https://candeltechservices.com/hvac-contractor-carrollton-tx/</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>services@candeltechservices.com</t>
@@ -6844,6 +6843,118 @@
         </is>
       </c>
       <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Arlington, TX Roofing Services – Relentless Contracting LLC</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>relentlesscontracting.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://relentlesscontracting.com/service-areas/arlington-tx</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>chris@relentlesscontracting.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>2148457663</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Arlington TX</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>90</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>roofing contractor Arlington TX</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Assist Roofing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>assistroofing.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.assistroofing.com/location-tampa-fl</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>sales@assistroofing.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>813-314-7950</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>88</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Tampa FL</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:18 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6869,7 +6869,6 @@
           <t>https://relentlesscontracting.com/service-areas/arlington-tx</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>chris@relentlesscontracting.com</t>
@@ -6925,7 +6924,6 @@
           <t>https://www.assistroofing.com/location-tampa-fl</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>sales@assistroofing.com</t>
@@ -6955,6 +6953,66 @@
         </is>
       </c>
       <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Jackson MS Roofing Contractor-  Gerardo's Construction</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>gerardosconstruction.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.gerardosconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Home Improvement</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@gerardosconstruction.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(601) 896-3983</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Jackson MS</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>100</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>roofing contractor Jackson MS</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:19 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7018,6 +7018,66 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Roofing in Gary, IN | Roof Repair &amp; Replacement | GRA</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>grageneralhomeservices.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://grageneralhomeservices.com/roofing-gary/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Services About</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>grageneralhomeservices@gmail.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>(708) 852-8357</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Gary IN</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>90</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>roof replacement Gary IN</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:24 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7078,6 +7078,62 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Local HVAC Company in Lafayette, LA | Freedom Air Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>freedomairlafayette.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.freedomairlafayette.com/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>freedomairhvac@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(337) 344-9920</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>90</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:29 UTC (cycle 173)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7099,7 +7099,6 @@
           <t>https://www.freedomairlafayette.com/</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>freedomairhvac@hotmail.com</t>
@@ -7129,6 +7128,66 @@
         </is>
       </c>
       <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Meridian Plumbing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>meridianinplumbing.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://meridianinplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Meridian These</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>usmanmaan302gb@gmail.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>(614) 756-0643</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Meridian ID</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>emergency plumber Meridian ID</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:31 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7193,6 +7193,62 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Plumbing Services | Duluth, MN | AquaTech Duluth Plumber</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>aquatechduluth.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://www.aquatechduluth.com/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>jadin@aquatechduluth.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>218-341-1596</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>90</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>plumbing company Duluth MN</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:32 UTC (cycle 175)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7214,7 +7214,6 @@
           <t>https://www.aquatechduluth.com/</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>jadin@aquatechduluth.com</t>
@@ -7244,6 +7243,66 @@
         </is>
       </c>
       <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Top-Rated Mechanical Contractor in Cedar Rapids, Iowa</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>mymoose.us</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://mymoose.us/services/water-heater-repair-replacement-in-cedar-rapids-iowa/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Moose Mechanical</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>brett.l@mymoose.us</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>319-440-9836</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>98</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>water heater repair Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:34 UTC (cycle 176)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7308,6 +7308,118 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Clearwater Roofing Company</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>roofing-clearwater.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.roofing-clearwater.com/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>john@gmail.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>(727) 472-9019</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>98</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>roofing contractor Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Drain Cleaning | Rapid City, SD</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>rcrapidrooter.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.rcrapidrooter.com/service</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>rcrapidrooter@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>(605) 220-7307</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Rapid City SD</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>86</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>drain cleaning service Rapid City SD</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:35 UTC (cycle 177)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7329,7 +7329,6 @@
           <t>https://www.roofing-clearwater.com/</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>john@gmail.com</t>
@@ -7385,7 +7384,6 @@
           <t>https://www.rcrapidrooter.com/service</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
           <t>rcrapidrooter@yahoo.com</t>
@@ -7415,6 +7413,66 @@
         </is>
       </c>
       <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Plumbers 911 Chicago</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>plumbers911chicago.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://plumbers911chicago.com/chicago-il-plumbing/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Why Chicago</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>info@plumbers911chicago.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>833-758-6911</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>100</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>drain cleaning service Chicago IL</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:46 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7478,6 +7478,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>American Custom Contractors</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>americancustomcontractors.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://americancustomcontractors.com/arlington-va/</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>President William</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>info@americancustomcontractors.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(301) 417-1000</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Arlington VA</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>90</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>roofing contractor Arlington VA</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:48 UTC (cycle 185)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7538,6 +7538,66 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Metal Roofing Salinas</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>ivansroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://ivansroofinginc.com/areas-of-service/salinas-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Commercial Roofing</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>contact@ivansroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(831) 307-1172</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>100</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Salinas CA</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:49 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7598,6 +7598,122 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Air Conditioning Installation &amp; Repair in NJ</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>mjmhvacnj.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://mjmhvacnj.com/air-conditioning</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Air Conditioning</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>mjmhvacnj@gmail.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(732) 366-4213</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>90</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>AC installation Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Quality HVAC and Refrigeration</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>qualityhvactx.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://www.qualityhvactx.com/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>info@qualityhvactx.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>(512) 738-0081</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>88</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>heating and cooling company San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-13 08:51 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7679,7 +7679,6 @@
           <t>https://www.qualityhvactx.com/</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>info@qualityhvactx.com</t>
@@ -7709,6 +7708,62 @@
         </is>
       </c>
       <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Hodge Mechanical</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>hodgemech.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://www.hodgemech.com/equipment-we-service/heat-pumps</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>service@hodgemech.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>(330) 205-2175</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Canton OH</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>90</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>heat pump installation Canton OH</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 09:02 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7734,7 +7734,6 @@
           <t>https://www.hodgemech.com/equipment-we-service/heat-pumps</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>service@hodgemech.com</t>
@@ -7764,6 +7763,126 @@
         </is>
       </c>
       <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Accurate Electric, Plumbing, Heating and Air</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>accurateelectricplumbingheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://accurateelectricplumbingheatingandair.com/service-area/rancho-cucamonga-ca/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Integrity Driven</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>info@accurateelectricplumbingheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>(626) 250-0051</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>100</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>air conditioning repair Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Peak Performance Roofing</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>peakperformanceroof.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://peakperformanceroof.com/service-area/hillsboro-or/</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Owens Corning</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>contact@wilsonmarketingco.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>971-979-7325</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>100</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>roof replacement Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-13 09:05 UTC (cycle 196)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-13.xlsx
+++ b/output/leads_2026-09-13.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7888,6 +7888,66 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Got Plumbing - Parma, OH</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>gotplumbingparma.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://gotplumbingparma.com/</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Got Plumbing</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>cmlurz@icloud.com</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>(440) 876-3702</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Parma OH</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>94</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>plumber Parma OH</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>